<commit_message>
update README on additional files
</commit_message>
<xml_diff>
--- a/input/MWI_metadata.xlsx
+++ b/input/MWI_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lwillem/Documents/university/other_projects/Xiao_rota/Rota_CEA_two-countries/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7575403-FCB8-6D4B-BF87-6DB637E54359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21067AD3-1E4E-7441-9EAB-B3EC258D5DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1980" yWindow="2600" windowWidth="26440" windowHeight="14660" xr2:uid="{0E11D85D-C1E7-1249-BC68-3B3C85704BA3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="49">
   <si>
     <t xml:space="preserve">Data from 2025 to 2034 </t>
   </si>
@@ -47,9 +47,6 @@
     <t xml:space="preserve">range of columns </t>
   </si>
   <si>
-    <t xml:space="preserve">moderate_to-sever case </t>
-  </si>
-  <si>
     <t>from column B to column GS</t>
   </si>
   <si>
@@ -81,9 +78,6 @@
   </si>
   <si>
     <t>from column PJ  to column PS</t>
-  </si>
-  <si>
-    <t>Sheet names</t>
   </si>
   <si>
     <t>novacc</t>
@@ -125,33 +119,6 @@
     </r>
   </si>
   <si>
-    <t>RV3BB_sch_longer_wv</t>
-  </si>
-  <si>
-    <t>switching to neonatal vaccine from 2025 –  for this duration of vaccine-induced immunity is doubling the variance of wv estimate for Rotavac from Ghana</t>
-  </si>
-  <si>
-    <t>RV3BB_sch_shorter_wv</t>
-  </si>
-  <si>
-    <t>switching to neonatal vaccine from 2025 –  for this duration of vaccine-induced immunity is doubling variance of wv estimate for Rotrix vaccine in Ghana</t>
-  </si>
-  <si>
-    <t>1_6_10_sch_double_wv_variance</t>
-  </si>
-  <si>
-    <t>switching to neonatal vaccine from 2025 –  for this duration of vaccine-induced immunity is doubling the variance of the model estimated rotarix vaccine induced immunity</t>
-  </si>
-  <si>
-    <t>6_10_14_rotavac_sc_wv</t>
-  </si>
-  <si>
-    <t>estimate using response rate and duration of vaccine-induced immunity from Ghana for rotavac vaccine</t>
-  </si>
-  <si>
-    <t>malawi_rotavac_6_10_14_dwRV1</t>
-  </si>
-  <si>
     <t>Rotavac: dw of Rotarix in MWI response rate and duration</t>
   </si>
   <si>
@@ -225,13 +192,34 @@
   </si>
   <si>
     <t>rotarix_6_10_14_sch</t>
+  </si>
+  <si>
+    <t>File names</t>
+  </si>
+  <si>
+    <t xml:space="preserve">moderate to sever cases </t>
+  </si>
+  <si>
+    <t>rv3bb_sampling_pooled_wv</t>
+  </si>
+  <si>
+    <t>opv_rv3bb_sampling_wv</t>
+  </si>
+  <si>
+    <t>rotavac_6_10_14_dwRV1</t>
+  </si>
+  <si>
+    <t>switching to neonatal vaccine from 2025 –  with pooled duration of vaccine-induced immunity</t>
+  </si>
+  <si>
+    <t>switching to neonatal vaccine from 2025 –  OPV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -244,6 +232,12 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -266,8 +260,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -602,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B218FDC3-9CA1-254F-B52B-17B766E7B16D}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="56.5" customWidth="1"/>
@@ -610,243 +605,227 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.15">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
       <c r="C3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
       <c r="C6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
+      <c r="A8" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.15">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A22" t="s">
         <v>25</v>
       </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A23" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.15">
-      <c r="A15" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A24" t="s">
         <v>27</v>
       </c>
-      <c r="B15" t="s">
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A25" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A17" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A26" t="s">
         <v>29</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A27" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A18" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A28" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A19" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A29" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A20" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A30" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A21" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A31" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A22" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A32" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A23" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A24" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A25" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A26" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A27" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A28" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A29" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A30" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A31" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A32" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A36" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A37" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>